<commit_message>
docs(ledger): R-064 검증대기 반영, R-065 신규 등록
- R-064 승인대기 → 검증대기 (32597b0). 1차 구현에서 itemCache 로 항목을 걸렀다가
  선택 항목의 상세만 들어 있어 표가 거의 안 걸러지던 것을 over_sigma 로 바꾼 경위를
  반영 내용에 남겼다
- R-065 신규 등록 → 검증대기 (ed65a85). 결과 탭 이름 변경과 탭 옆 숫자 제거
- 안내 §5 이력에 2026-10-19 한 줄

신뢰성툴 65건 = 완료 42 / 검증대기 23 (승인대기 0)

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MezXSHa6eeUcgNLHojHfgZ
</commit_message>
<xml_diff>
--- a/docs/요구사항관리대장.xlsx
+++ b/docs/요구사항관리대장.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="379">
   <si>
     <t xml:space="preserve">요구사항 관리 대장</t>
   </si>
@@ -4173,6 +4173,417 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">그대로다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026-10-19 — R-064 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">반영</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(32597b0): </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">요약 배지 카드를 누르면 그 유형의 데이터만 보기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">표</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그래프 동반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차 구현에서 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">itemCache </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 항목을 걸렀다가 선택 항목의 상세만 들어 있어 표가 거의 안 걸러지는 것을 확인하고 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">over_sigma </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 바꿨다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. R-065 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">반영</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(ed65a85): </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">결과 탭 이름을 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'Fail </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">분석 결과</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'/'Pass </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">분석 결과</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 바꾸고 탭 옆 숫자 제거</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">신뢰성툴 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">65</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">건 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">42 / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">검증대기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">23. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기본값은 여전히 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">legacy, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴리즈 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Rev.0.031 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그대로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미푸시 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">13</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">커밋</t>
     </r>
     <r>
       <rPr>
@@ -15877,6 +16288,210 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">filteredResultRows() </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">체인에 유형 필터를 한 겹 얹어 표</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">드롭박스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그래프가 한 자리에서 모두 따라오게 했다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(R-054 Item </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">검색과 같은 지점</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">둘은 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AND). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유형별 샘플 집합은 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">R-053 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">unitTypeSetsByCondition() </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">을 그대로 쓴다 — 신뢰성 항목</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·FT Temp </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">필터를 이미 타고 있어 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Fail </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">탭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(Fail Type)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">과 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Pass </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">탭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">(</t>
     </r>
     <r>
@@ -15885,7 +16500,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">미착수</t>
+      <t xml:space="preserve">셀렉 유형</t>
     </r>
     <r>
       <rPr>
@@ -15902,24 +16517,279 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">확정된 사양</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">: filteredResultRows() </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">체인에 유형 필터를 한 겹 얹어 표</t>
+      <t xml:space="preserve">양쪽에 통한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. ※ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">항목 판정은 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">over_sigma </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 한다 — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">itemCache </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 선택한 항목의 상세만 들고 있어서 그걸로 보면 나머지 항목이 전부 통과해 표가 거의 안 걸러진다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차 구현에서 실제로 그랬다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). over_sigma </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 샘플마다 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그 샘플이 걸린 항목 목록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">을 들고 전 항목을 덮는다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">카드별</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유형 카드→그 유형만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, '</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">총 진행</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'/'Pass </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">진행</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">해제</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, '</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">벤치 검토 필요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제외 유형</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(Tail·Unstable)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">을 뺀 전부</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">재클릭 해제</t>
     </r>
     <r>
       <rPr>
@@ -15936,7 +16806,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">드롭박스</t>
+      <t xml:space="preserve">다른 카드 전환</t>
     </r>
     <r>
       <rPr>
@@ -15953,24 +16823,41 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">그래프가 자동으로 따라오게 한다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(R-054 Item </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">검색과 같은 자리</t>
+      <t xml:space="preserve">선택 카드 음영과 하단 강조선</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">탭을 옮기면 푼다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">두 탭은 유형 이름 자체가 다르다</t>
     </r>
     <r>
       <rPr>
@@ -15987,24 +16874,24 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">어떤 샘플이 그 유형인지는 기존 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">unitTypeSetsByCondition() </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">을 쓴다 — 신뢰성 항목</t>
+      <t xml:space="preserve">유형별 샘플 집합은 한 번 그릴 때 한 번만 만들고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">항목</t>
     </r>
     <r>
       <rPr>
@@ -16021,92 +16908,24 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">온도 필터를 이미 타고 있어 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Fail </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">탭</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(Fail Type)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">과 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Abnormal Pass </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">탭</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">셀렉 유형</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">양쪽에 통한다</t>
+      <t xml:space="preserve">온도 필터가 바뀌면 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">renderSummary() </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에서 버린다</t>
     </r>
     <r>
       <rPr>
@@ -16123,126 +16942,24 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">카드별</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">유형 카드→그 유형만</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, '</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">총 진행</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'/'Pass </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">진행</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'→</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">해제</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, '</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">벤치 검토 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'→</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제외 유형을 뺀 전부</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">재클릭 해제</t>
+      <t xml:space="preserve">표시 전용 — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">payload·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">캐시 스키마</t>
     </r>
     <r>
       <rPr>
@@ -16259,241 +16976,244 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">다른 카드 전환</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">선택 카드 음영</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">경계</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">보던 항목이 필터에 안 걸리면 첫 항목으로 이동</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(R-054 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">와 같은 규칙</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">), </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">탭 전환 시 해제</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">유형 이름이 다르다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">), 0</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">건이면 안내</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, Item </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">검색과 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">AND. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">표시 전용 — </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">payload·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">캐시 스키마</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">판정 미변경</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">배지 숫자는 필터와 무관하게 유지한다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">필터로 숫자가 변하면 기준을 잃는다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">).</t>
+      <t xml:space="preserve">판정 미변경이고 배지 숫자도 필터와 무관하게 유지한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Eden 님 요청 2026-10-17. 사전 보고 완료, 착수 대기.</t>
+    <t xml:space="preserve">32597b0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eden 님 요청 2026-10-17. 검증(Playwright · Test Data SM3502Q · shape 모드): 샘플 기준 표 22행 → Excessive 3행(#25·#75·#79) / Separated 19행 / 벤치 검토 필요 22행, 해제하면 22행 복귀. 선택 항목 상세도 그 유형 행만. 탭 전환 시 해제 확인. 콘솔 에러 없음. 게이트 PASS(단위 3건 + 골든 회귀 2/2).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R-065</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">결과 탭 명칭을 바꾸고 탭 이름 옆 숫자를 없앨 것 — 'Fail 항목' → 'Fail 분석 결과', 'Abnormal Pass' → 'Pass 분석 결과'.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">탭 두 개의 라벨을 바꾸고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">탭 이름 옆에 붙던 숫자 배지를 뺐다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">바로 아래 배지 카드가 같은 값을 더 크게 보여주고 있어 군더더기였고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">둘의 단위가 달라</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">탭 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이상 항목 수 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">배지 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유닛 수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">같은 자리에 다른 숫자가 보이는 꼴이라 오히려 헷갈렸다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">옛 창이나 되돌린 상태에서 배지 노드가 남아 있을 수 있어 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">renderSummaryStrip() </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에서 지우고 시작한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. setTabBadge() </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 다른 곳에서 쓸 수 있게 남겨 뒀다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">ed65a85</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eden 님 요청 2026-10-19. 표시 전용. 게이트 PASS(단위 3건 + 골든 회귀 2/2), 콘솔 에러 없음.</t>
   </si>
   <si>
     <t xml:space="preserve">E-001</t>
@@ -17336,7 +18056,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -17430,6 +18150,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -17781,7 +18505,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
@@ -17839,7 +18563,7 @@
       </c>
       <c r="D6" s="8" t="n">
         <f aca="false">COUNTIF(신뢰성툴!D:D,"승인대기")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="8" t="n">
         <f aca="false">COUNTIF(신뢰성툴!D:D,"작업중")</f>
@@ -17847,7 +18571,7 @@
       </c>
       <c r="F6" s="8" t="n">
         <f aca="false">COUNTIF(신뢰성툴!D:D,"검증대기")</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G6" s="8" t="n">
         <f aca="false">COUNTIF(신뢰성툴!D:D,"완료")</f>
@@ -18231,9 +18955,14 @@
         <v>63</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="21" t="s">
         <v>64</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="21" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -18304,1472 +19033,1488 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G3" s="22"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G4" s="22" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G5" s="22"/>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G6" s="22"/>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G7" s="22"/>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G9" s="22"/>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G11" s="22" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G17" s="22" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G18" s="22" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G19" s="22" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G20" s="22" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G21" s="22" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G22" s="22" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G23" s="22" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G24" s="22" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G25" s="22" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G26" s="22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C27" s="22" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G27" s="22" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G30" s="22" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G31" s="22" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G32" s="22" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G33" s="22" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E34" s="22" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G34" s="22" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G35" s="22" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E36" s="22" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G36" s="22" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="8" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="G37" s="22" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="8" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E38" s="22" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G38" s="22" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E39" s="22" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="G39" s="22" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="8" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E40" s="22" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="G40" s="22" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="8" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E41" s="22" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G41" s="22" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="8" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E42" s="22" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G42" s="22" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="8" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E43" s="22" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="G43" s="22" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="8" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D44" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G44" s="22" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="8" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G45" s="22" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="8" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F46" s="8" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G46" s="22" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C47" s="22" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E47" s="22" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G47" s="22" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="8" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D48" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G48" s="22" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="8" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G49" s="22" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="8" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D50" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G50" s="22" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="8" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G51" s="22" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="8" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C52" s="22" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D52" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E52" s="23" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G52" s="22" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="8" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C53" s="22" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E53" s="23" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G53" s="22" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="8" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D54" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E54" s="22" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G54" s="22" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="8" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C55" s="22" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E55" s="23" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G55" s="22" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="8" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C56" s="22" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D56" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E56" s="22" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F56" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G56" s="22" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="8" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C57" s="22" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E57" s="22" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F57" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G57" s="22" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="8" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C58" s="22" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D58" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E58" s="22" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F58" s="8" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G58" s="22" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="8" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C59" s="22" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E59" s="23" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G59" s="22" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="8" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C60" s="22" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D60" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E60" s="23" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F60" s="8" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G60" s="22" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="8" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C61" s="22" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E61" s="23" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F61" s="8" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G61" s="22" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="8" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C62" s="22" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D62" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E62" s="23" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F62" s="8" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G62" s="22" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="8" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C63" s="22" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D63" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E63" s="23" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="F63" s="8" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G63" s="22" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="8" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D64" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E64" s="23" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F64" s="8" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G64" s="22" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="8" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B65" s="8" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E65" s="23" t="s">
-        <v>360</v>
-      </c>
-      <c r="F65" s="8"/>
+        <v>361</v>
+      </c>
+      <c r="F65" s="8" t="s">
+        <v>362</v>
+      </c>
       <c r="G65" s="22" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="8"/>
-      <c r="B66" s="8"/>
-      <c r="C66" s="22"/>
-      <c r="D66" s="6"/>
-      <c r="E66" s="22"/>
-      <c r="F66" s="8"/>
-      <c r="G66" s="22"/>
+      <c r="A66" s="8" t="s">
+        <v>364</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="C66" s="22" t="s">
+        <v>366</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E66" s="24" t="s">
+        <v>367</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="G66" s="22" t="s">
+        <v>369</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="8"/>
@@ -26528,23 +27273,23 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="F2" s="8"/>
       <c r="G2" s="22" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33880,23 +34625,23 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="F2" s="8"/>
       <c r="G2" s="23" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
docs(ledger): R-061·R-062·R-063 완료 — shape 를 기본 판정 모드로 릴리즈
Eden 님이 실데이터로 shape 이상 없음을 확인했고, Rev.0.033(v0.0.33)으로 기본값이
되어 나가므로 실질 승인이다. 세 건 모두 F열에 커밋 해시가 있어 완료 조건을 만족한다
(안내 §3 — 해시 없으면 완료로 바꾸지 않는다).

- R-061 완료 (53a322b) · R-062·R-063 완료 (766a857)
- 비고에 완료 경위를 남겼다 — 리비전을 나눠 legacy(Rev.0.032)도 같이 내보내는 것,
  게이트가 두 모드를 각각 대조하는 것, 화면에 Tail=legacy/shape 가 찍히는 것
- 안내 §5 이력에 릴리즈 둘(v0.0.32 · v0.0.33) 한 줄

신뢰성툴 65건 = 완료 45 / 검증대기 20 (R-043~R-060, R-064·R-065)

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MezXSHa6eeUcgNLHojHfgZ
</commit_message>
<xml_diff>
--- a/docs/요구사항관리대장.xlsx
+++ b/docs/요구사항관리대장.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="380">
   <si>
     <t xml:space="preserve">요구사항 관리 대장</t>
   </si>
@@ -4584,6 +4584,284 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">커밋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026-10-19 (2) — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴리즈 둘</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. Rev.0.032(v0.0.32) = legacy, Rev.0.033(v0.0.33) = shape. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">코드는 같고 기본 판정 모드만 다르며</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, exe </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이름이 리비전을 달고 나와 파일명으로 구분된다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. R-061·R-062·R-063 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">을 완료로 올렸다 — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">shape </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 기본값으로 내보내는 것이 실질 승인이다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">게이트가 두 모드를 각각 대조하도록 고쳤고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(tests/golden_shape/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">신설</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, run_checks </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가 환경변수로 모드를 명시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">), test_retest_history </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도 두 모드를 모두 고정한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">게이트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">PASS 5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">건</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">남은 검증대기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">건</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(R-043~R-060, R-064·R-065)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 그대로다</t>
     </r>
     <r>
       <rPr>
@@ -15345,7 +15623,7 @@
     <t xml:space="preserve">766a857</t>
   </si>
   <si>
-    <t xml:space="preserve">Eden 님 지시 2026-10-17 (11.202 FT_7V_-9p8V_PH1_900mA_Min, HTOL Room 500hrs 그래프). 실데이터(Test Data 조건x항목 1003) 전후: Separated-&gt;Tail 188항목/상세 614, Tail-&gt;Separated 0. ※ 지시 항목 자체는 하한 쪽이 구제(z=2.26 &lt; 3.65)되지만, 같은 항목 상한 쪽에 0.8007(Excessive) 유닛이 있어 항목 판정을 상·하한 중 보수적인 쪽으로 합치는 규칙 때문에 여전히 Separated — 쪽별 판정 분리 여부 결정 대기. 측정(실데이터 전 조건, 중복 제외 · R-061 → R-061+062+063): Separated 363→213, Tail 346→496. 전이는 Separated→Tail 150 쌍 한 방향뿐(구제형). 벤치 검토 필요 130→121 유닛. 게이트 PASS(단위 3건 + 골든 회귀 2/2) — legacy 불변.</t>
+    <t xml:space="preserve">Eden 님 지시 2026-10-17 (11.202 FT_7V_-9p8V_PH1_900mA_Min, HTOL Room 500hrs 그래프). 실데이터(Test Data 조건x항목 1003) 전후: Separated-&gt;Tail 188항목/상세 614, Tail-&gt;Separated 0. ※ 지시 항목 자체는 하한 쪽이 구제(z=2.26 &lt; 3.65)되지만, 같은 항목 상한 쪽에 0.8007(Excessive) 유닛이 있어 항목 판정을 상·하한 중 보수적인 쪽으로 합치는 규칙 때문에 여전히 Separated — 쪽별 판정 분리 여부 결정 대기. 측정(실데이터 전 조건, 중복 제외 · R-061 → R-061+062+063): Separated 363→213, Tail 346→496. 전이는 Separated→Tail 150 쌍 한 방향뿐(구제형). 벤치 검토 필요 130→121 유닛. 게이트 PASS(단위 3건 + 골든 회귀 2/2) — legacy 불변. [완료 2026-10-19] Eden 님이 실데이터로 shape 이상 없음을 확인해 기본 판정 모드로 올렸다. Rev.0.033(v0.0.33)으로 릴리즈하며, legacy 는 Rev.0.032(v0.0.32)로 같이 내보낸다 — 판정이 바뀌는 변경이라 리비전을 나눴다(CLAUDE.md §5-1). 게이트도 두 모드를 각각 대조하도록 고쳤다(tests/golden/ · tests/golden_shape/). 화면 상단과 시작 배너에 Tail=legacy / Tail=shape 가 찍힌다.</t>
   </si>
   <si>
     <t xml:space="preserve">R-063</t>
@@ -15535,7 +15813,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Eden 님 지시 2026-10-17. 계기: 11.202 FT_7V_-9p8V_PH1_900mA_Min (HTOL Room 500hrs) — 하한 쪽 3유닛은 R-062 구제로 Tail 인데 상한 쪽 +0.8007 유닛(Excessive) 때문에 항목 판정이 Separated 로 묶였다. 규격 안 유닛은 판정 대상이 아니다(Eden 님 확인). | 검증 2026-10-17 (Test Data, shape 모드, Excessive 우선 적용): fail 상세행 R-062→R-063 Separated→Tail 30건, 역방향 0건 / 유닛(가장 심한 유형) Separated→Tail 8유닛. 바뀐 항목은 HTOL 500hrs Room 의 -10V/-9.8V PH1 계열 5항목×2폴더뿐. 11.202 항목은 서버 API 로 하한 이탈 3유닛 Tail, 상한 +0.8007 유닛 Excessive 확인. legacy regression PASS 2/2. 측정(실데이터 전 조건, 중복 제외 · R-061 → R-061+062+063): Separated 363→213, Tail 346→496. 전이는 Separated→Tail 150 쌍 한 방향뿐(구제형). 벤치 검토 필요 130→121 유닛. 게이트 PASS(단위 3건 + 골든 회귀 2/2) — legacy 불변.</t>
+    <t xml:space="preserve">Eden 님 지시 2026-10-17. 계기: 11.202 FT_7V_-9p8V_PH1_900mA_Min (HTOL Room 500hrs) — 하한 쪽 3유닛은 R-062 구제로 Tail 인데 상한 쪽 +0.8007 유닛(Excessive) 때문에 항목 판정이 Separated 로 묶였다. 규격 안 유닛은 판정 대상이 아니다(Eden 님 확인). | 검증 2026-10-17 (Test Data, shape 모드, Excessive 우선 적용): fail 상세행 R-062→R-063 Separated→Tail 30건, 역방향 0건 / 유닛(가장 심한 유형) Separated→Tail 8유닛. 바뀐 항목은 HTOL 500hrs Room 의 -10V/-9.8V PH1 계열 5항목×2폴더뿐. 11.202 항목은 서버 API 로 하한 이탈 3유닛 Tail, 상한 +0.8007 유닛 Excessive 확인. legacy regression PASS 2/2. 측정(실데이터 전 조건, 중복 제외 · R-061 → R-061+062+063): Separated 363→213, Tail 346→496. 전이는 Separated→Tail 150 쌍 한 방향뿐(구제형). 벤치 검토 필요 130→121 유닛. 게이트 PASS(단위 3건 + 골든 회귀 2/2) — legacy 불변. [완료 2026-10-19] Eden 님이 실데이터로 shape 이상 없음을 확인해 기본 판정 모드로 올렸다. Rev.0.033(v0.0.33)으로 릴리즈하며, legacy 는 Rev.0.032(v0.0.32)로 같이 내보낸다 — 판정이 바뀌는 변경이라 리비전을 나눴다(CLAUDE.md §5-1). 게이트도 두 모드를 각각 대조하도록 고쳤다(tests/golden/ · tests/golden_shape/). 화면 상단과 시작 배너에 Tail=legacy / Tail=shape 가 찍힌다.</t>
   </si>
   <si>
     <t xml:space="preserve">R-061</t>
@@ -16272,7 +16550,7 @@
     <t xml:space="preserve">53a322b</t>
   </si>
   <si>
-    <t xml:space="preserve">양자화 임계 근거: 511 (조건×항목) 의 σ_core/분해능이 0(40건) · 1.48(17건) · 2.97(11건) 에 몰려 있다가 3.71 에서 1 건으로 끊긴다 — MAD 가 분해능의 정수배라 1.4826×k 로만 나온다. 임계 4 로 올려도 1 건만 늘어 둔감. 측정(실데이터 전 조건, 중복 제외 · legacy→shape): Intermittent 1→0, Unstable 6→1, Slight 43→0, Shift 0(양자화 제외로 전부 사라짐), Separated 0→363, Tail 662→346. 벤치 검토 필요 102→130 유닛. 게이트 PASS(단위 3건 + 골든 회귀 2/2) — legacy 불변. ※ 기본값 전환 여부는 미정.</t>
+    <t xml:space="preserve">양자화 임계 근거: 511 (조건×항목) 의 σ_core/분해능이 0(40건) · 1.48(17건) · 2.97(11건) 에 몰려 있다가 3.71 에서 1 건으로 끊긴다 — MAD 가 분해능의 정수배라 1.4826×k 로만 나온다. 임계 4 로 올려도 1 건만 늘어 둔감. 측정(실데이터 전 조건, 중복 제외 · legacy→shape): Intermittent 1→0, Unstable 6→1, Slight 43→0, Shift 0(양자화 제외로 전부 사라짐), Separated 0→363, Tail 662→346. 벤치 검토 필요 102→130 유닛. 게이트 PASS(단위 3건 + 골든 회귀 2/2) — legacy 불변. ※ 기본값 전환 여부는 미정. [완료 2026-10-19] Eden 님이 실데이터로 shape 이상 없음을 확인해 기본 판정 모드로 올렸다. Rev.0.033(v0.0.33)으로 릴리즈하며, legacy 는 Rev.0.032(v0.0.32)로 같이 내보낸다 — 판정이 바뀌는 변경이라 리비전을 나눴다(CLAUDE.md §5-1). 게이트도 두 모드를 각각 대조하도록 고쳤다(tests/golden/ · tests/golden_shape/). 화면 상단과 시작 배너에 Tail=legacy / Tail=shape 가 찍힌다.</t>
   </si>
   <si>
     <t xml:space="preserve">R-064</t>
@@ -17004,210 +17282,7 @@
     <t xml:space="preserve">결과 탭 명칭을 바꾸고 탭 이름 옆 숫자를 없앨 것 — 'Fail 항목' → 'Fail 분석 결과', 'Abnormal Pass' → 'Pass 분석 결과'.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">탭 두 개의 라벨을 바꾸고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">탭 이름 옆에 붙던 숫자 배지를 뺐다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">바로 아래 배지 카드가 같은 값을 더 크게 보여주고 있어 군더더기였고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">둘의 단위가 달라</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">탭 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">= </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이상 항목 수 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">배지 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">= </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">유닛 수</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">같은 자리에 다른 숫자가 보이는 꼴이라 오히려 헷갈렸다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">옛 창이나 되돌린 상태에서 배지 노드가 남아 있을 수 있어 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">renderSummaryStrip() </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">에서 지우고 시작한다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. setTabBadge() </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">는 다른 곳에서 쓸 수 있게 남겨 뒀다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
+    <t xml:space="preserve">탭 두 개의 라벨을 바꾸고, 탭 이름 옆에 붙던 숫자 배지를 뺐다. 바로 아래 배지 카드가 같은 값을 더 크게 보여주고 있어 군더더기였고, 둘의 단위가 달라(탭 = 이상 항목 수 / 배지 = 유닛 수) 같은 자리에 다른 숫자가 보이는 꼴이라 오히려 헷갈렸다. 옛 창이나 되돌린 상태에서 배지 노드가 남아 있을 수 있어 renderSummaryStrip() 에서 지우고 시작한다. setTabBadge() 는 다른 곳에서 쓸 수 있게 남겨 뒀다.</t>
   </si>
   <si>
     <t xml:space="preserve">ed65a85</t>
@@ -18056,7 +18131,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -18150,10 +18225,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -18505,7 +18576,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
@@ -18571,11 +18642,11 @@
       </c>
       <c r="F6" s="8" t="n">
         <f aca="false">COUNTIF(신뢰성툴!D:D,"검증대기")</f>
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G6" s="8" t="n">
         <f aca="false">COUNTIF(신뢰성툴!D:D,"완료")</f>
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18960,9 +19031,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="21" t="s">
         <v>65</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="21" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -19033,1487 +19109,1487 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G3" s="22"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G4" s="22" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G5" s="22"/>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G6" s="22"/>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G7" s="22"/>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G9" s="22"/>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G11" s="22" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G17" s="22" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G18" s="22" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G19" s="22" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G20" s="22" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G21" s="22" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G22" s="22" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G23" s="22" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G24" s="22" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G25" s="22" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G26" s="22" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C27" s="22" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G27" s="22" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G30" s="22" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G31" s="22" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G32" s="22" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G33" s="22" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E34" s="22" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G34" s="22" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G35" s="22" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E36" s="22" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G36" s="22" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="8" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="G37" s="22" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="8" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E38" s="22" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="G38" s="22" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E39" s="22" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G39" s="22" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="8" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E40" s="22" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G40" s="22" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="8" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E41" s="22" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G41" s="22" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="8" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E42" s="22" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G42" s="22" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="8" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E43" s="22" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G43" s="22" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="8" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D44" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="G44" s="22" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="8" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="G45" s="22" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="8" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F46" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="G46" s="22" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C47" s="22" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E47" s="22" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G47" s="22" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D48" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G48" s="22" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="8" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G49" s="22" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="8" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D50" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G50" s="22" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="8" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G51" s="22" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="8" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C52" s="22" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D52" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E52" s="23" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G52" s="22" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="8" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C53" s="22" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E53" s="23" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G53" s="22" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="8" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D54" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E54" s="22" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G54" s="22" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="8" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C55" s="22" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E55" s="23" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G55" s="22" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="8" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C56" s="22" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D56" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E56" s="22" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F56" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G56" s="22" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="8" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C57" s="22" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E57" s="22" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F57" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G57" s="22" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="8" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C58" s="22" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D58" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E58" s="22" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F58" s="8" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G58" s="22" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="8" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C59" s="22" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E59" s="23" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G59" s="22" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="8" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C60" s="22" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D60" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E60" s="23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F60" s="8" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G60" s="22" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="8" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C61" s="22" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E61" s="23" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F61" s="8" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G61" s="22" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="8" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C62" s="22" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E62" s="23" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F62" s="8" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G62" s="22" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="8" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C63" s="22" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E63" s="23" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F63" s="8" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G63" s="22" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="8" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E64" s="23" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F64" s="8" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G64" s="22" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="8" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B65" s="8" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D65" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E65" s="23" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F65" s="8" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="G65" s="22" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="8" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C66" s="22" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D66" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E66" s="24" t="s">
-        <v>367</v>
+      <c r="E66" s="22" t="s">
+        <v>368</v>
       </c>
       <c r="F66" s="8" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G66" s="22" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27273,23 +27349,23 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F2" s="8"/>
       <c r="G2" s="22" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -34625,23 +34701,23 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F2" s="8"/>
       <c r="G2" s="23" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>